<commit_message>
Update template: Summary sheet is now the first visible sheet
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/templates/TPR_IP_Template.xlsx
+++ b/templates/TPR_IP_Template.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Bayona\Python\Projects\tpr-ip-viz\tpr-ip-viz\templates\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Pamela Bayona\Documents\Python Projects\tpr-ip-viz\templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5DD21E3F-1ED8-4068-9AE1-54FCDFE480B1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="1000" firstSheet="2" activeTab="10" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="5895" yWindow="5595" windowWidth="28800" windowHeight="13065" tabRatio="1000" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Summary" sheetId="5" r:id="rId1"/>

</xml_diff>